<commit_message>
set up SWMM and TRITON-only benchmarking test cases
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_swmm.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_swmm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECAEFC9C-8C00-4929-AB95-1C97A3DCCB62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{111BC0A2-D04B-4FD8-96FA-4EE3C48A48A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="18">
   <si>
     <t>CPU</t>
   </si>
@@ -90,9 +90,6 @@
   </si>
   <si>
     <t>standard</t>
-  </si>
-  <si>
-    <t>hpc_time_min_per_sim</t>
   </si>
 </sst>
 </file>
@@ -314,7 +311,7 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
@@ -337,9 +334,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Input" xfId="1" builtinId="20"/>
@@ -347,7 +341,7 @@
     <cellStyle name="Note" xfId="3" builtinId="10"/>
     <cellStyle name="Output" xfId="2" builtinId="21"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="16">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -414,25 +408,6 @@
         <horizontal style="thin">
           <color indexed="64"/>
         </horizontal>
-      </border>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
       </border>
     </dxf>
     <dxf>
@@ -676,23 +651,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1A4495C6-64F1-4654-82C3-1417CFDBC1D1}" name="Table1" displayName="Table1" ref="A1:M8" totalsRowShown="0" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14" totalsRowBorderDxfId="13">
-  <autoFilter ref="A1:M8" xr:uid="{1A4495C6-64F1-4654-82C3-1417CFDBC1D1}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1A4495C6-64F1-4654-82C3-1417CFDBC1D1}" name="Table1" displayName="Table1" ref="A1:L8" totalsRowShown="0" headerRowDxfId="15" headerRowBorderDxfId="14" tableBorderDxfId="13" totalsRowBorderDxfId="12">
+  <autoFilter ref="A1:L8" xr:uid="{1A4495C6-64F1-4654-82C3-1417CFDBC1D1}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L8">
     <sortCondition ref="E1:E8"/>
   </sortState>
-  <tableColumns count="13">
-    <tableColumn id="11" xr3:uid="{3DECB62C-AAF2-4EC7-8598-5E8776D4B845}" name="hardware_utilization_strategy" dataDxfId="12" dataCellStyle="Note"/>
-    <tableColumn id="9" xr3:uid="{047B8296-C28F-43DA-A753-CC6445B34CE4}" name="device" dataDxfId="11" dataCellStyle="Note"/>
-    <tableColumn id="1" xr3:uid="{16000747-EB63-4EDF-971B-D9460636B6A5}" name="run_mode" dataDxfId="10" dataCellStyle="Input"/>
-    <tableColumn id="2" xr3:uid="{09DC1F4B-B2B0-493A-B83E-1D7D4EA31F4C}" name="n_nodes" dataDxfId="9" dataCellStyle="Input"/>
-    <tableColumn id="3" xr3:uid="{3A65E5E5-CB8B-4698-A27C-21DF3A95D49A}" name="n_mpi_procs" dataDxfId="8" dataCellStyle="Input"/>
-    <tableColumn id="4" xr3:uid="{D366E835-7967-45B3-94DD-92B04C3126AA}" name="n_omp_threads" dataDxfId="7" dataCellStyle="Input"/>
-    <tableColumn id="8" xr3:uid="{53D9FE6F-92F7-4A3A-B94F-6A698F029BE0}" name="n_gpus" dataDxfId="6" dataCellStyle="Input"/>
-    <tableColumn id="12" xr3:uid="{97D9BCE9-C2EB-487D-9081-3F6B6CACB117}" name="hpc_ensemble_partition" dataDxfId="5" dataCellStyle="Input"/>
-    <tableColumn id="13" xr3:uid="{96650528-E8C5-445B-8564-B12E25175139}" name="hpc_time_min_per_sim" dataDxfId="4" dataCellStyle="Input">
-      <calculatedColumnFormula>60*6</calculatedColumnFormula>
-    </tableColumn>
+  <tableColumns count="12">
+    <tableColumn id="11" xr3:uid="{3DECB62C-AAF2-4EC7-8598-5E8776D4B845}" name="hardware_utilization_strategy" dataDxfId="11" dataCellStyle="Note"/>
+    <tableColumn id="9" xr3:uid="{047B8296-C28F-43DA-A753-CC6445B34CE4}" name="device" dataDxfId="10" dataCellStyle="Note"/>
+    <tableColumn id="1" xr3:uid="{16000747-EB63-4EDF-971B-D9460636B6A5}" name="run_mode" dataDxfId="9" dataCellStyle="Input"/>
+    <tableColumn id="2" xr3:uid="{09DC1F4B-B2B0-493A-B83E-1D7D4EA31F4C}" name="n_nodes" dataDxfId="8" dataCellStyle="Input"/>
+    <tableColumn id="3" xr3:uid="{3A65E5E5-CB8B-4698-A27C-21DF3A95D49A}" name="n_mpi_procs" dataDxfId="7" dataCellStyle="Input"/>
+    <tableColumn id="4" xr3:uid="{D366E835-7967-45B3-94DD-92B04C3126AA}" name="n_omp_threads" dataDxfId="6" dataCellStyle="Input"/>
+    <tableColumn id="8" xr3:uid="{53D9FE6F-92F7-4A3A-B94F-6A698F029BE0}" name="n_gpus" dataDxfId="5" dataCellStyle="Input"/>
+    <tableColumn id="12" xr3:uid="{97D9BCE9-C2EB-487D-9081-3F6B6CACB117}" name="hpc_ensemble_partition" dataDxfId="4" dataCellStyle="Input"/>
     <tableColumn id="6" xr3:uid="{F6B7A6B4-BD4B-4406-BCB7-C3DBCC48FA6B}" name="total_OpenMP_threads" dataDxfId="3" dataCellStyle="Output">
       <calculatedColumnFormula>Table1[[#This Row],[n_mpi_procs]]*Table1[[#This Row],[n_omp_threads]]</calculatedColumnFormula>
     </tableColumn>
@@ -973,7 +945,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.85546875" bestFit="1" customWidth="1"/>
@@ -982,13 +954,13 @@
     <col min="4" max="4" width="19" customWidth="1"/>
     <col min="5" max="5" width="22.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="28.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="9" width="28.28515625" customWidth="1"/>
-    <col min="10" max="10" width="24.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19" customWidth="1"/>
-    <col min="12" max="12" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="28.28515625" customWidth="1"/>
+    <col min="9" max="9" width="24.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="19" customWidth="1"/>
+    <col min="11" max="11" width="19.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1013,23 +985,20 @@
       <c r="H1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="12" t="s">
-        <v>18</v>
+      <c r="I1" s="2" t="s">
+        <v>6</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
@@ -1054,28 +1023,24 @@
       <c r="H2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="4">
-        <f>60*6</f>
-        <v>360</v>
+      <c r="I2" s="5">
+        <f>Table1[[#This Row],[n_mpi_procs]]*Table1[[#This Row],[n_omp_threads]]</f>
+        <v>1</v>
       </c>
       <c r="J2" s="5">
-        <f>Table1[[#This Row],[n_mpi_procs]]*Table1[[#This Row],[n_omp_threads]]</f>
-        <v>1</v>
-      </c>
-      <c r="K2" s="5">
         <f>Table1[[#This Row],[n_omp_threads]]*Table1[[#This Row],[n_mpi_procs]]</f>
         <v>1</v>
       </c>
-      <c r="L2" s="6">
+      <c r="K2" s="6">
         <f>Table1[[#This Row],[total_devices]]/Table1[[#This Row],[n_nodes]]</f>
         <v>1</v>
       </c>
-      <c r="M2" t="b">
+      <c r="L2" t="b">
         <f>Table1[[#This Row],[n_mpi_procs]]&gt;=Table1[[#This Row],[n_nodes]]</f>
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>2</v>
       </c>
@@ -1100,28 +1065,24 @@
       <c r="H3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I3" s="4">
-        <f>60*6</f>
-        <v>360</v>
-      </c>
-      <c r="J3" s="5">
+      <c r="I3" s="5">
         <f>Table1[[#This Row],[n_mpi_procs]]*Table1[[#This Row],[n_omp_threads]]</f>
         <v>2</v>
       </c>
-      <c r="K3" s="5">
+      <c r="J3" s="5">
         <f>Table1[[#This Row],[n_omp_threads]]*Table1[[#This Row],[n_mpi_procs]]</f>
         <v>2</v>
       </c>
-      <c r="L3" s="6">
+      <c r="K3" s="6">
         <f>Table1[[#This Row],[total_devices]]/Table1[[#This Row],[n_nodes]]</f>
         <v>2</v>
       </c>
-      <c r="M3" t="b">
+      <c r="L3" t="b">
         <f>Table1[[#This Row],[n_mpi_procs]]&gt;=Table1[[#This Row],[n_nodes]]</f>
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
@@ -1146,28 +1107,24 @@
       <c r="H4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I4" s="4">
-        <f>60*6</f>
-        <v>360</v>
-      </c>
-      <c r="J4" s="5">
+      <c r="I4" s="5">
         <f>Table1[[#This Row],[n_mpi_procs]]*Table1[[#This Row],[n_omp_threads]]</f>
         <v>4</v>
       </c>
-      <c r="K4" s="5">
+      <c r="J4" s="5">
         <f>Table1[[#This Row],[n_omp_threads]]*Table1[[#This Row],[n_mpi_procs]]</f>
         <v>4</v>
       </c>
-      <c r="L4" s="6">
+      <c r="K4" s="6">
         <f>Table1[[#This Row],[total_devices]]/Table1[[#This Row],[n_nodes]]</f>
         <v>4</v>
       </c>
-      <c r="M4" t="b">
+      <c r="L4" t="b">
         <f>Table1[[#This Row],[n_mpi_procs]]&gt;=Table1[[#This Row],[n_nodes]]</f>
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>2</v>
       </c>
@@ -1192,28 +1149,24 @@
       <c r="H5" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="4">
-        <f>60*6</f>
-        <v>360</v>
-      </c>
-      <c r="J5" s="5">
+      <c r="I5" s="5">
         <f>Table1[[#This Row],[n_mpi_procs]]*Table1[[#This Row],[n_omp_threads]]</f>
         <v>8</v>
       </c>
-      <c r="K5" s="5">
+      <c r="J5" s="5">
         <f>Table1[[#This Row],[n_omp_threads]]*Table1[[#This Row],[n_mpi_procs]]</f>
         <v>8</v>
       </c>
-      <c r="L5" s="6">
+      <c r="K5" s="6">
         <f>Table1[[#This Row],[total_devices]]/Table1[[#This Row],[n_nodes]]</f>
         <v>8</v>
       </c>
-      <c r="M5" t="b">
+      <c r="L5" t="b">
         <f>Table1[[#This Row],[n_mpi_procs]]&gt;=Table1[[#This Row],[n_nodes]]</f>
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
         <v>2</v>
       </c>
@@ -1238,28 +1191,24 @@
       <c r="H6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I6" s="4">
-        <f>60*6</f>
-        <v>360</v>
-      </c>
-      <c r="J6" s="5">
+      <c r="I6" s="5">
         <f>Table1[[#This Row],[n_mpi_procs]]*Table1[[#This Row],[n_omp_threads]]</f>
         <v>16</v>
       </c>
-      <c r="K6" s="5">
+      <c r="J6" s="5">
         <f>Table1[[#This Row],[n_omp_threads]]*Table1[[#This Row],[n_mpi_procs]]</f>
         <v>16</v>
       </c>
-      <c r="L6" s="6">
+      <c r="K6" s="6">
         <f>Table1[[#This Row],[total_devices]]/Table1[[#This Row],[n_nodes]]</f>
         <v>16</v>
       </c>
-      <c r="M6" t="b">
+      <c r="L6" t="b">
         <f>Table1[[#This Row],[n_mpi_procs]]&gt;=Table1[[#This Row],[n_nodes]]</f>
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>2</v>
       </c>
@@ -1284,28 +1233,24 @@
       <c r="H7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I7" s="4">
-        <f>60*6</f>
-        <v>360</v>
-      </c>
-      <c r="J7" s="5">
+      <c r="I7" s="5">
         <f>Table1[[#This Row],[n_mpi_procs]]*Table1[[#This Row],[n_omp_threads]]</f>
         <v>32</v>
       </c>
-      <c r="K7" s="5">
+      <c r="J7" s="5">
         <f>Table1[[#This Row],[n_omp_threads]]*Table1[[#This Row],[n_mpi_procs]]</f>
         <v>32</v>
       </c>
-      <c r="L7" s="6">
+      <c r="K7" s="6">
         <f>Table1[[#This Row],[total_devices]]/Table1[[#This Row],[n_nodes]]</f>
         <v>32</v>
       </c>
-      <c r="M7" t="b">
+      <c r="L7" t="b">
         <f>Table1[[#This Row],[n_mpi_procs]]&gt;=Table1[[#This Row],[n_nodes]]</f>
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
         <v>2</v>
       </c>
@@ -1330,23 +1275,19 @@
       <c r="H8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="I8" s="4">
-        <f>60*6</f>
-        <v>360</v>
-      </c>
-      <c r="J8" s="5">
+      <c r="I8" s="5">
         <f>Table1[[#This Row],[n_mpi_procs]]*Table1[[#This Row],[n_omp_threads]]</f>
         <v>64</v>
       </c>
-      <c r="K8" s="5">
+      <c r="J8" s="5">
         <f>Table1[[#This Row],[n_omp_threads]]*Table1[[#This Row],[n_mpi_procs]]</f>
         <v>64</v>
       </c>
-      <c r="L8" s="6">
+      <c r="K8" s="6">
         <f>Table1[[#This Row],[total_devices]]/Table1[[#This Row],[n_nodes]]</f>
         <v>64</v>
       </c>
-      <c r="M8" t="b">
+      <c r="L8" t="b">
         <f>Table1[[#This Row],[n_mpi_procs]]&gt;=Table1[[#This Row],[n_nodes]]</f>
         <v>1</v>
       </c>

</xml_diff>